<commit_message>
chore: update release package to v1.0.0, rebuild all assets
- Regenerate 01_产品介绍.pdf, 02_样例报告.html/pdf, 03_使用说明.pdf
- Regenerate 04_示例数据.xlsx, 06_常见问题.pdf
- Replace 05_试用版安装包.zip with ML-Diagnostic-Tool-v1.0.0.zip
- Add *.zip to .gitignore for release package
</commit_message>
<xml_diff>
--- a/发布包/04_示例数据.xlsx
+++ b/发布包/04_示例数据.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="混凝土强度数据" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="混凝土强度数据" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>